<commit_message>
refactor: 统一为 date./form. 两种 Sheet 类型
</commit_message>
<xml_diff>
--- a/data/报告数据.xlsx
+++ b/data/报告数据.xlsx
@@ -7,9 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_全局信息" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="data.shareholders" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="data.shareholder_info" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="date.全局信息" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="form.股东出资" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="form.股东信息" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -437,7 +437,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>g.company_name</t>
+          <t>date.公司名</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -449,7 +449,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>g.credit_code</t>
+          <t>date.信用代码</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -461,7 +461,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>g.registered_address</t>
+          <t>date.注册地址</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -473,7 +473,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>g.legal_representative</t>
+          <t>date.法定代表人</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -485,7 +485,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>g.company_type</t>
+          <t>date.公司类型</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -497,7 +497,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>g.registered_capital</t>
+          <t>date.注册资本</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -507,7 +507,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>g.business_scope</t>
+          <t>date.经营范围</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -519,7 +519,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>g.established_date</t>
+          <t>date.成立日期</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -531,7 +531,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>g.operating_period</t>
+          <t>date.经营期限</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -564,27 +564,27 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>shareholder_name</t>
+          <t>股东</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>subscribed_amount</t>
+          <t>认缴金额</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>subscribed_ratio</t>
+          <t>认缴比例</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>paid_amount</t>
+          <t>实缴金额</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>paid_ratio</t>
+          <t>实缴比例</t>
         </is>
       </c>
     </row>
@@ -666,12 +666,12 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>序号</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>detail</t>
+          <t>详情</t>
         </is>
       </c>
     </row>

</xml_diff>